<commit_message>
Fix group-by demo: Revenue was already numeric, making tonumber a no-op
Confirmed directly: sales.xlsx's Revenue column used SetCellValue with
a native Go int, so it was already a genuine numeric cell - tonumber
on it did nothing, which contradicted the hero demo's own "text needs
tonumber" lesson right next to it on the same page. Regenerated the
fixture with Revenue stored as text instead (the same real-world
export quirk the hero's Likes column has), re-verified both the
without-tonumber case now errors the same way the hero's does and the
with-tonumber case still totals correctly (1500/1250/150, unchanged),
and re-rendered the GIF.
</commit_message>
<xml_diff>
--- a/docs/vhs/fixtures/sales.xlsx
+++ b/docs/vhs/fixtures/sales.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Category</t>
   </si>
@@ -25,10 +25,25 @@
     <t>Shoes</t>
   </si>
   <si>
+    <t>1200</t>
+  </si>
+  <si>
     <t>Shirts</t>
   </si>
   <si>
+    <t>850</t>
+  </si>
+  <si>
+    <t>300</t>
+  </si>
+  <si>
     <t>Hats</t>
+  </si>
+  <si>
+    <t>150</t>
+  </si>
+  <si>
+    <t>400</t>
   </si>
 </sst>
 </file>
@@ -347,40 +362,40 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2">
-        <v>1200</v>
+      <c r="B2" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>850</v>
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
         <v>2</v>
       </c>
-      <c r="B4">
-        <v>300</v>
+      <c r="B4" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>150</v>
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6">
-        <v>400</v>
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>